<commit_message>
Update recruitment data for 2026-08-04
</commit_message>
<xml_diff>
--- a/2027届秋招投递信息_2026-07-24.xlsx
+++ b/2027届秋招投递信息_2026-07-24.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前开放项目" sheetId="1" r:id="R749d57a1ba014186"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="近期明确截止" sheetId="2" r:id="R7f0c4d5993cd48f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与统计" sheetId="3" r:id="Rc853f8092b164847"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前开放项目" sheetId="1" r:id="Rd3b867ef39d04225"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="近期明确截止" sheetId="2" r:id="R8f9b3003bfa1476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与统计" sheetId="3" r:id="R011f61f9abfc4d52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -705,7 +705,7 @@
         <x:v>南大就业公众号文章发布于2026-08-01，面向2027届毕业生（毕业时间为2026年9月至2027年8月），工作地点为深圳、上海、珠海；简历投递截止2026-10-31 19:00，8-11月安排笔面试、10月起沟通Offer。岗位城市和具体职位以影石Insta360官方招聘页为准。</x:v>
       </x:c>
       <x:c r="O4" s="15" t="str">
-        <x:v>https://www.insta360.com/cn/jobs</x:v>
+        <x:v>https://mp.weixin.qq.com/s?__biz=MzAxMDA3MjIwMw==&amp;mid=2652174609&amp;idx=1&amp;sn=341a17d61257a145a21e44df7633757a&amp;chksm=81427f5412a5949a05987cdd3b7c4a6d9bea8bd715ad941339cf4c6373e216476c4fc00456a7&amp;scene=27</x:v>
       </x:c>
       <x:c r="P4" s="14" t="str">
         <x:v>A-企业官方招聘页与官方公众号文章交叉核验</x:v>
@@ -6209,7 +6209,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35b243dc075e4fec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54cd0616e22f43a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7006,7 +7006,7 @@
         <x:v>南大就业公众号文章发布于2026-08-01，面向2027届毕业生（毕业时间为2026年9月至2027年8月），工作地点为深圳、上海、珠海；简历投递截止2026-10-31 19:00，8-11月安排笔面试、10月起沟通Offer。岗位城市和具体职位以影石Insta360官方招聘页为准。</x:v>
       </x:c>
       <x:c r="O16" s="15" t="str">
-        <x:v>https://www.insta360.com/cn/jobs</x:v>
+        <x:v>https://mp.weixin.qq.com/s?__biz=MzAxMDA3MjIwMw==&amp;mid=2652174609&amp;idx=1&amp;sn=341a17d61257a145a21e44df7633757a&amp;chksm=81427f5412a5949a05987cdd3b7c4a6d9bea8bd715ad941339cf4c6373e216476c4fc00456a7&amp;scene=27</x:v>
       </x:c>
       <x:c r="P16" s="14" t="str">
         <x:v>A-企业官方招聘页与官方公众号文章交叉核验</x:v>
@@ -7234,7 +7234,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R949de6a5a1fa4261"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26a1d8c8a7414a7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>